<commit_message>
Beginning of Smoke Test Cases creation + Implementation
</commit_message>
<xml_diff>
--- a/E-Commerce Web/Amazon/Test Suites/Functional Testing Suite/Smoke Tests.xlsx
+++ b/E-Commerce Web/Amazon/Test Suites/Functional Testing Suite/Smoke Tests.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="47">
   <si>
     <t>Test Case ID</t>
   </si>
@@ -48,13 +48,118 @@
     <t>Comments</t>
   </si>
   <si>
-    <t>1.</t>
-  </si>
-  <si>
-    <t>2.</t>
-  </si>
-  <si>
-    <t>3.</t>
+    <t>Status (Mobile)</t>
+  </si>
+  <si>
+    <t>Test Case Data</t>
+  </si>
+  <si>
+    <t>TC-SMK-1</t>
+  </si>
+  <si>
+    <t>Registration</t>
+  </si>
+  <si>
+    <t>Positive</t>
+  </si>
+  <si>
+    <t>TC-SMK-2</t>
+  </si>
+  <si>
+    <t>Negative</t>
+  </si>
+  <si>
+    <t>1. Choose new account registration</t>
+  </si>
+  <si>
+    <t>Email: takimawot555@gmail.com Password: 1234</t>
+  </si>
+  <si>
+    <t>2. Enter email address, name and password</t>
+  </si>
+  <si>
+    <t>1. Entering the Amazon main page  2. Click on Sign In button (top, right)</t>
+  </si>
+  <si>
+    <t>Error message about password (must be more than 6 letters)</t>
+  </si>
+  <si>
+    <t>Passed</t>
+  </si>
+  <si>
+    <t>The web site do not react on wrong email</t>
+  </si>
+  <si>
+    <t>3. Input wrong password verification</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Error message about wrong password matching </t>
+  </si>
+  <si>
+    <t>TC-SMK-3</t>
+  </si>
+  <si>
+    <t>Email: takimawot555@gmail.com Password: 123456</t>
+  </si>
+  <si>
+    <t>Email: takimawot@gmail.com Password: 123456</t>
+  </si>
+  <si>
+    <t>Successful registration</t>
+  </si>
+  <si>
+    <t>Sign In</t>
+  </si>
+  <si>
+    <t>TC-SMK-4</t>
+  </si>
+  <si>
+    <t>1. Entering the Amazon main page  2. Sign out (if account is signed in)</t>
+  </si>
+  <si>
+    <t>Verification of application reaction on invalid inputs for registration</t>
+  </si>
+  <si>
+    <t>Verification of application reaction on valid inputs for registration</t>
+  </si>
+  <si>
+    <t>Verification of application reaction on invalid password for signing in</t>
+  </si>
+  <si>
+    <t>1. Write the email address</t>
+  </si>
+  <si>
+    <t>2. Wait until password entering line appears</t>
+  </si>
+  <si>
+    <t>3. Enter wrong password</t>
+  </si>
+  <si>
+    <t>Email: takimawot@gmail.com Password: 213456</t>
+  </si>
+  <si>
+    <t>Error message about incorrect password</t>
+  </si>
+  <si>
+    <t>TC-SMK-5</t>
+  </si>
+  <si>
+    <t>3. Enter password</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Successful log in </t>
+  </si>
+  <si>
+    <t>Log In</t>
+  </si>
+  <si>
+    <t>1. Entering the Amazon main page  2. Sign out (if account is logged in)</t>
+  </si>
+  <si>
+    <t>Verification of application reaction on invalid password for logging in</t>
+  </si>
+  <si>
+    <t>Verification of application reaction on valid password for logging in</t>
   </si>
 </sst>
 </file>
@@ -142,22 +247,46 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
@@ -438,87 +567,485 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="B2:J5"/>
+  <dimension ref="A1:K21"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="11.5546875" customWidth="1"/>
+    <col min="2" max="2" width="12.88671875" customWidth="1"/>
+    <col min="3" max="3" width="13.109375" customWidth="1"/>
+    <col min="4" max="4" width="30" customWidth="1"/>
+    <col min="5" max="5" width="30.109375" customWidth="1"/>
+    <col min="6" max="6" width="36.77734375" customWidth="1"/>
+    <col min="7" max="7" width="28.44140625" customWidth="1"/>
+    <col min="8" max="8" width="26.88671875" customWidth="1"/>
+    <col min="9" max="9" width="7.5546875" customWidth="1"/>
+    <col min="10" max="10" width="13.77734375" customWidth="1"/>
+    <col min="11" max="11" width="18.21875" customWidth="1"/>
+    <col min="13" max="13" width="10.109375" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="2" spans="2:10" x14ac:dyDescent="0.3">
-      <c r="B2" s="1" t="s">
+    <row r="1" spans="1:11" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="F2" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="G2" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="H2" s="1" t="s">
+      <c r="G1" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="H1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="I2" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="J2" s="1" t="s">
+      <c r="J1" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="1" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="2:10" x14ac:dyDescent="0.3">
-      <c r="B3" s="2"/>
-      <c r="C3" s="2"/>
-      <c r="D3" s="3"/>
-      <c r="E3" s="2"/>
-      <c r="F3" s="2"/>
-      <c r="G3" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="H3" s="2"/>
-      <c r="I3" s="2"/>
-      <c r="J3" s="2"/>
-    </row>
-    <row r="4" spans="2:10" x14ac:dyDescent="0.3">
-      <c r="B4" s="4"/>
-      <c r="C4" s="4"/>
-      <c r="D4" s="3"/>
-      <c r="E4" s="4"/>
-      <c r="F4" s="4"/>
-      <c r="G4" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="H4" s="4"/>
-      <c r="I4" s="4"/>
-      <c r="J4" s="4"/>
-    </row>
-    <row r="5" spans="2:10" x14ac:dyDescent="0.3">
-      <c r="B5" s="5"/>
-      <c r="C5" s="5"/>
-      <c r="D5" s="3"/>
-      <c r="E5" s="5"/>
-      <c r="F5" s="5"/>
-      <c r="G5" s="6" t="s">
+    <row r="2" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="H5" s="5"/>
-      <c r="I5" s="5"/>
-      <c r="J5" s="5"/>
+      <c r="B2" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="C2" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="F2" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="G2" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="H2" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="I2" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="J2" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="K2" s="4" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" ht="19.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="11"/>
+      <c r="B3" s="11"/>
+      <c r="C3" s="11"/>
+      <c r="D3" s="7"/>
+      <c r="E3" s="7"/>
+      <c r="F3" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="G3" s="11"/>
+      <c r="H3" s="7"/>
+      <c r="I3" s="11"/>
+      <c r="J3" s="11"/>
+      <c r="K3" s="7"/>
+    </row>
+    <row r="4" spans="1:11" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="B4" s="13" t="s">
+        <v>12</v>
+      </c>
+      <c r="C4" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="D4" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="E4" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="G4" s="13" t="s">
+        <v>26</v>
+      </c>
+      <c r="H4" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="I4" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="J4" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="K4" s="6"/>
+    </row>
+    <row r="5" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="13"/>
+      <c r="B5" s="13"/>
+      <c r="C5" s="13"/>
+      <c r="D5" s="6"/>
+      <c r="E5" s="6"/>
+      <c r="F5" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="G5" s="13"/>
+      <c r="H5" s="6"/>
+      <c r="I5" s="13"/>
+      <c r="J5" s="13"/>
+      <c r="K5" s="6"/>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A6" s="13"/>
+      <c r="B6" s="13"/>
+      <c r="C6" s="13"/>
+      <c r="D6" s="6"/>
+      <c r="E6" s="6"/>
+      <c r="F6" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="G6" s="13"/>
+      <c r="H6" s="6"/>
+      <c r="I6" s="13"/>
+      <c r="J6" s="13"/>
+      <c r="K6" s="6"/>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A7" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="B7" s="13" t="s">
+        <v>12</v>
+      </c>
+      <c r="C7" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="D7" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="E7" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="F7" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="G7" s="13" t="s">
+        <v>27</v>
+      </c>
+      <c r="H7" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="I7" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="J7" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="K7" s="6"/>
+    </row>
+    <row r="8" spans="1:11" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="13"/>
+      <c r="B8" s="13"/>
+      <c r="C8" s="13"/>
+      <c r="D8" s="6"/>
+      <c r="E8" s="6"/>
+      <c r="F8" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="G8" s="13"/>
+      <c r="H8" s="6"/>
+      <c r="I8" s="13"/>
+      <c r="J8" s="13"/>
+      <c r="K8" s="6"/>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A9" s="13"/>
+      <c r="B9" s="13"/>
+      <c r="C9" s="13"/>
+      <c r="D9" s="6"/>
+      <c r="E9" s="6"/>
+      <c r="F9" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="G9" s="13"/>
+      <c r="H9" s="6"/>
+      <c r="I9" s="13"/>
+      <c r="J9" s="13"/>
+      <c r="K9" s="6"/>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A10" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="B10" s="10" t="s">
+        <v>43</v>
+      </c>
+      <c r="C10" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="D10" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="E10" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="F10" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="G10" s="13" t="s">
+        <v>38</v>
+      </c>
+      <c r="H10" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="I10" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="J10" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="K10" s="4"/>
+    </row>
+    <row r="11" spans="1:11" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="11"/>
+      <c r="B11" s="11"/>
+      <c r="C11" s="11"/>
+      <c r="D11" s="7"/>
+      <c r="E11" s="7"/>
+      <c r="F11" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="G11" s="13"/>
+      <c r="H11" s="7"/>
+      <c r="I11" s="11"/>
+      <c r="J11" s="11"/>
+      <c r="K11" s="7"/>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A12" s="12"/>
+      <c r="B12" s="12"/>
+      <c r="C12" s="12"/>
+      <c r="D12" s="8"/>
+      <c r="E12" s="8"/>
+      <c r="F12" s="9" t="s">
+        <v>37</v>
+      </c>
+      <c r="G12" s="13"/>
+      <c r="H12" s="8"/>
+      <c r="I12" s="12"/>
+      <c r="J12" s="12"/>
+      <c r="K12" s="8"/>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A13" s="10" t="s">
+        <v>40</v>
+      </c>
+      <c r="B13" s="10" t="s">
+        <v>43</v>
+      </c>
+      <c r="C13" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="D13" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="E13" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="F13" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="G13" s="13" t="s">
+        <v>27</v>
+      </c>
+      <c r="H13" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="I13" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="J13" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="K13" s="4"/>
+    </row>
+    <row r="14" spans="1:11" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="11"/>
+      <c r="B14" s="11"/>
+      <c r="C14" s="11"/>
+      <c r="D14" s="7"/>
+      <c r="E14" s="7"/>
+      <c r="F14" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="G14" s="13"/>
+      <c r="H14" s="7"/>
+      <c r="I14" s="11"/>
+      <c r="J14" s="11"/>
+      <c r="K14" s="7"/>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A15" s="12"/>
+      <c r="B15" s="12"/>
+      <c r="C15" s="12"/>
+      <c r="D15" s="8"/>
+      <c r="E15" s="8"/>
+      <c r="F15" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="G15" s="13"/>
+      <c r="H15" s="8"/>
+      <c r="I15" s="12"/>
+      <c r="J15" s="12"/>
+      <c r="K15" s="8"/>
+    </row>
+    <row r="19" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A19" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="B19" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="C19" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="D19" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="E19" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="F19" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="G19" s="13" t="s">
+        <v>38</v>
+      </c>
+      <c r="H19" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="I19" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="J19" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="K19" s="4"/>
+    </row>
+    <row r="20" spans="1:11" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A20" s="11"/>
+      <c r="B20" s="11"/>
+      <c r="C20" s="11"/>
+      <c r="D20" s="7"/>
+      <c r="E20" s="7"/>
+      <c r="F20" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="G20" s="13"/>
+      <c r="H20" s="7"/>
+      <c r="I20" s="11"/>
+      <c r="J20" s="11"/>
+      <c r="K20" s="7"/>
+    </row>
+    <row r="21" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A21" s="12"/>
+      <c r="B21" s="12"/>
+      <c r="C21" s="12"/>
+      <c r="D21" s="8"/>
+      <c r="E21" s="8"/>
+      <c r="F21" s="9" t="s">
+        <v>37</v>
+      </c>
+      <c r="G21" s="13"/>
+      <c r="H21" s="8"/>
+      <c r="I21" s="12"/>
+      <c r="J21" s="12"/>
+      <c r="K21" s="8"/>
     </row>
   </sheetData>
-  <mergeCells count="8">
-    <mergeCell ref="I3:I5"/>
-    <mergeCell ref="J3:J5"/>
-    <mergeCell ref="B3:B5"/>
-    <mergeCell ref="C3:C5"/>
-    <mergeCell ref="D3:D5"/>
-    <mergeCell ref="E3:E5"/>
-    <mergeCell ref="F3:F5"/>
-    <mergeCell ref="H3:H5"/>
+  <mergeCells count="60">
+    <mergeCell ref="J13:J15"/>
+    <mergeCell ref="K13:K15"/>
+    <mergeCell ref="D13:D15"/>
+    <mergeCell ref="E13:E15"/>
+    <mergeCell ref="G13:G15"/>
+    <mergeCell ref="H13:H15"/>
+    <mergeCell ref="I13:I15"/>
+    <mergeCell ref="K7:K9"/>
+    <mergeCell ref="A10:A12"/>
+    <mergeCell ref="B10:B12"/>
+    <mergeCell ref="C10:C12"/>
+    <mergeCell ref="D10:D12"/>
+    <mergeCell ref="E10:E12"/>
+    <mergeCell ref="G10:G12"/>
+    <mergeCell ref="H10:H12"/>
+    <mergeCell ref="I10:I12"/>
+    <mergeCell ref="J10:J12"/>
+    <mergeCell ref="K10:K12"/>
+    <mergeCell ref="E7:E9"/>
+    <mergeCell ref="G7:G9"/>
+    <mergeCell ref="H7:H9"/>
+    <mergeCell ref="I7:I9"/>
+    <mergeCell ref="J7:J9"/>
+    <mergeCell ref="E4:E6"/>
+    <mergeCell ref="G4:G6"/>
+    <mergeCell ref="H4:H6"/>
+    <mergeCell ref="I4:I6"/>
+    <mergeCell ref="J4:J6"/>
+    <mergeCell ref="K4:K6"/>
+    <mergeCell ref="K19:K21"/>
+    <mergeCell ref="E2:E3"/>
+    <mergeCell ref="A2:A3"/>
+    <mergeCell ref="B2:B3"/>
+    <mergeCell ref="C2:C3"/>
+    <mergeCell ref="D2:D3"/>
+    <mergeCell ref="G2:G3"/>
+    <mergeCell ref="H2:H3"/>
+    <mergeCell ref="I2:I3"/>
+    <mergeCell ref="J2:J3"/>
+    <mergeCell ref="K2:K3"/>
+    <mergeCell ref="E19:E21"/>
+    <mergeCell ref="G19:G21"/>
+    <mergeCell ref="H19:H21"/>
+    <mergeCell ref="I19:I21"/>
+    <mergeCell ref="J19:J21"/>
+    <mergeCell ref="A19:A21"/>
+    <mergeCell ref="B19:B21"/>
+    <mergeCell ref="C19:C21"/>
+    <mergeCell ref="D19:D21"/>
+    <mergeCell ref="A4:A6"/>
+    <mergeCell ref="B4:B6"/>
+    <mergeCell ref="C4:C6"/>
+    <mergeCell ref="D4:D6"/>
+    <mergeCell ref="A7:A9"/>
+    <mergeCell ref="B7:B9"/>
+    <mergeCell ref="C7:C9"/>
+    <mergeCell ref="D7:D9"/>
+    <mergeCell ref="A13:A15"/>
+    <mergeCell ref="B13:B15"/>
+    <mergeCell ref="C13:C15"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>